<commit_message>
Defined the SavingsAccount Class and fixed some minor typos on other files. Also setup for Unit Test Plan for Savings Account
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_savings_account.xlsx
+++ b/tests/A02_pixell_test_plan_savings_account.xlsx
@@ -1,35 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Updated Assignments ISD\assignment_02\given_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keith\Desktop\RRC_Polytech\Winter2025\SoftwareDevFiles_Intermediate\project\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E5394E5-D09B-4C82-AD73-79542EE783C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ECC0B46-B94B-4F94-BAAE-52F220F8DBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="25185" windowHeight="13845" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -161,14 +150,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
       <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
         </ext>
       </extLst>
@@ -183,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -233,9 +222,6 @@
     <t>balance less than minimum balance</t>
   </si>
   <si>
-    <t>Student Name</t>
-  </si>
-  <si>
     <t>Attributes are set to parameter values.</t>
   </si>
   <si>
@@ -246,6 +232,64 @@
   </si>
   <si>
     <t>balance  equal to minimum balance</t>
+  </si>
+  <si>
+    <t>Keith Robles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account Number must be numeric, Client Number must be numeric, date value is valid, balance must be a float, and minimum balance must be numeric.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_number = int, client_number = int, date = date(year, month, day)(numeric), balance = float, and minimum_balance = float
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is Valid with no errors raised and minimum balance is not set to 50.00
+</t>
+  </si>
+  <si>
+    <t>Minimum Balance is not numeric</t>
+  </si>
+  <si>
+    <t>not an int or float</t>
+  </si>
+  <si>
+    <t>sets Minimum Balance to 50.00</t>
+  </si>
+  <si>
+    <t>Minimum Balance is greater than Balance</t>
+  </si>
+  <si>
+    <t>Minium Balance is a lower float value than Balance</t>
+  </si>
+  <si>
+    <t>Service Charge is set to Base Service Charge</t>
+  </si>
+  <si>
+    <t>Minimum Balance is equal to the Balance</t>
+  </si>
+  <si>
+    <t>Minium Balance is a float value  equal to Balance</t>
+  </si>
+  <si>
+    <t>Minimum Balance is less than Balance</t>
+  </si>
+  <si>
+    <t>Minimum Balance is a lower float value than Balance</t>
+  </si>
+  <si>
+    <t>Correct Attributes</t>
+  </si>
+  <si>
+    <t>Attributes are correctly implemented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service Charge is set to Base Service Charge multiplied by Service Charge Premium </t>
+  </si>
+  <si>
+    <t>Prints out the following Example: Account Number: 9483914 Balance: $1,559.49
+Minimum Balance: $50.00 Account Type: Savings</t>
   </si>
 </sst>
 </file>
@@ -552,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -607,6 +651,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1179,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="18"/>
     </row>
@@ -1223,11 +1273,17 @@
         <v>8</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+        <v>16</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
@@ -1239,9 +1295,15 @@
       <c r="D8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
+      <c r="E8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
@@ -1251,11 +1313,17 @@
         <v>13</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+        <v>18</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
@@ -1265,11 +1333,17 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+        <v>19</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
@@ -1281,9 +1355,15 @@
       <c r="D11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11">
@@ -1293,11 +1373,17 @@
         <v>11</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="11">
@@ -1307,7 +1393,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
+      <c r="G13" s="24"/>
     </row>
     <row r="14" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
@@ -1517,9 +1603,10 @@
     <mergeCell ref="B34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>